<commit_message>
add w4a8 standard test script
</commit_message>
<xml_diff>
--- a/test/moe_w4a8/moegemmoutput.xlsx
+++ b/test/moe_w4a8/moegemmoutput.xlsx
@@ -465,10 +465,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C2" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D2" t="n">
         <v>7168</v>
@@ -477,7 +477,7 @@
         <v>128</v>
       </c>
       <c r="F2" t="n">
-        <v>101.3335226178169</v>
+        <v>175.3528115749359</v>
       </c>
     </row>
     <row r="3">
@@ -485,10 +485,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C3" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D3" t="n">
         <v>7168</v>
@@ -497,7 +497,7 @@
         <v>128</v>
       </c>
       <c r="F3" t="n">
-        <v>109.2696785926819</v>
+        <v>219.2783713340759</v>
       </c>
     </row>
     <row r="4">
@@ -505,10 +505,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C4" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D4" t="n">
         <v>7168</v>
@@ -517,7 +517,7 @@
         <v>128</v>
       </c>
       <c r="F4" t="n">
-        <v>113.0487197637558</v>
+        <v>279.8338308334351</v>
       </c>
     </row>
     <row r="5">
@@ -525,10 +525,10 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C5" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D5" t="n">
         <v>7168</v>
@@ -537,7 +537,7 @@
         <v>128</v>
       </c>
       <c r="F5" t="n">
-        <v>122.8847048282623</v>
+        <v>381.1367781162262</v>
       </c>
     </row>
     <row r="6">
@@ -545,10 +545,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C6" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D6" t="n">
         <v>7168</v>
@@ -557,7 +557,7 @@
         <v>128</v>
       </c>
       <c r="F6" t="n">
-        <v>125.6008620262146</v>
+        <v>547.3856072425842</v>
       </c>
     </row>
     <row r="7">
@@ -565,10 +565,10 @@
         <v>32</v>
       </c>
       <c r="B7" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C7" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D7" t="n">
         <v>7168</v>
@@ -577,7 +577,7 @@
         <v>128</v>
       </c>
       <c r="F7" t="n">
-        <v>133.2302922010422</v>
+        <v>774.2194976806641</v>
       </c>
     </row>
     <row r="8">
@@ -585,10 +585,10 @@
         <v>64</v>
       </c>
       <c r="B8" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C8" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D8" t="n">
         <v>7168</v>
@@ -597,7 +597,7 @@
         <v>128</v>
       </c>
       <c r="F8" t="n">
-        <v>151.4104385375977</v>
+        <v>996.8063478469849</v>
       </c>
     </row>
     <row r="9">
@@ -605,10 +605,10 @@
         <v>128</v>
       </c>
       <c r="B9" t="n">
-        <v>256</v>
+        <v>512</v>
       </c>
       <c r="C9" t="n">
-        <v>7168</v>
+        <v>3584</v>
       </c>
       <c r="D9" t="n">
         <v>7168</v>
@@ -617,7 +617,7 @@
         <v>128</v>
       </c>
       <c r="F9" t="n">
-        <v>171.7801847457886</v>
+        <v>1141.25967502594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add w4a8 marlin decode size1~1024 without streamk
</commit_message>
<xml_diff>
--- a/test/moe_w4a8/moegemmoutput.xlsx
+++ b/test/moe_w4a8/moegemmoutput.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,7 +477,7 @@
         <v>128</v>
       </c>
       <c r="F2" t="n">
-        <v>175.3528115749359</v>
+        <v>176.6326223611832</v>
       </c>
     </row>
     <row r="3">
@@ -497,7 +497,7 @@
         <v>128</v>
       </c>
       <c r="F3" t="n">
-        <v>219.2783713340759</v>
+        <v>216.555303812027</v>
       </c>
     </row>
     <row r="4">
@@ -517,7 +517,7 @@
         <v>128</v>
       </c>
       <c r="F4" t="n">
-        <v>279.8338308334351</v>
+        <v>270.7208487987518</v>
       </c>
     </row>
     <row r="5">
@@ -537,7 +537,7 @@
         <v>128</v>
       </c>
       <c r="F5" t="n">
-        <v>381.1367781162262</v>
+        <v>374.3791460990906</v>
       </c>
     </row>
     <row r="6">
@@ -557,7 +557,7 @@
         <v>128</v>
       </c>
       <c r="F6" t="n">
-        <v>547.3856072425842</v>
+        <v>530.7474579811096</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
         <v>128</v>
       </c>
       <c r="F7" t="n">
-        <v>774.2194976806641</v>
+        <v>745.0216155052185</v>
       </c>
     </row>
     <row r="8">
@@ -597,7 +597,7 @@
         <v>128</v>
       </c>
       <c r="F8" t="n">
-        <v>996.8063478469849</v>
+        <v>953.8610429763794</v>
       </c>
     </row>
     <row r="9">
@@ -617,7 +617,167 @@
         <v>128</v>
       </c>
       <c r="F9" t="n">
-        <v>1141.25967502594</v>
+        <v>2063.189926147461</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>256</v>
+      </c>
+      <c r="B10" t="n">
+        <v>512</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E10" t="n">
+        <v>128</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2117.086996078491</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>512</v>
+      </c>
+      <c r="B11" t="n">
+        <v>512</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E11" t="n">
+        <v>128</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2199.582654953003</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B12" t="n">
+        <v>512</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E12" t="n">
+        <v>128</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2372.581453323364</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2048</v>
+      </c>
+      <c r="B13" t="n">
+        <v>512</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E13" t="n">
+        <v>128</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2769.867593765259</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4096</v>
+      </c>
+      <c r="B14" t="n">
+        <v>512</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E14" t="n">
+        <v>128</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4349.436935424805</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6144</v>
+      </c>
+      <c r="B15" t="n">
+        <v>512</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D15" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E15" t="n">
+        <v>128</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5982.090805053711</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8192</v>
+      </c>
+      <c r="B16" t="n">
+        <v>512</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E16" t="n">
+        <v>128</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7607.159385681152</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16384</v>
+      </c>
+      <c r="B17" t="n">
+        <v>512</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7168</v>
+      </c>
+      <c r="E17" t="n">
+        <v>128</v>
+      </c>
+      <c r="F17" t="n">
+        <v>14151.56507873535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>